<commit_message>
feat(experiments): backfill 32-vocab mechanism contrast 438-445 into Excel
- 加法实验总表.xlsx: 32-vocab rows 438-445 with real 40Q scores
  (LSD 10/40, 雪崩 32/40, Looped4 27/40, Looped7 26/40, 验算 31/40...)
- builder: inject V32 measured rows keyed by mechanism id (438-445), add
  row id field; mechanism params auto-inferred from titles (lsd/looped/
  avalanche/carry_curriculum/self_verify/use_ans_tags)
- additive -> bfd14b4 (configs completed + params)
</commit_message>
<xml_diff>
--- a/迷宫实验总表.xlsx
+++ b/迷宫实验总表.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="全部迷宫实验总表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部迷宫实验总表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>